<commit_message>
feat(eval): consolida 10 modelos candidatos baixados e dataset de benchmark de imagem
- Atualiza backend/eval/model_benchmark/modelos.json e documentações com o pool de 10 modelos
  baixados no Ollama (Llama 3.2 11B Vision, Qwen2.5-VL 7B/3B, Qwen3.5 9B Q4/Defiant MTP,
  DeepSeek-R1-Distill-Llama-8B Q8, Phi-4-mini BF16, Gemma-3-Gaia 4B F16, Gemma-4-12B/E4B)
- Sincroniza modelos_ia_previstos (.csv, .xlsx, .md) e documentos (ARCHITECTURE, ROADMAP, EVALUATION)
- Monta dataset de benchmark de imagem com 72 casos e suporte a positivas sem aceitos manuais
- Adiciona contagem detalhada de tokens e custos de visão em OpenRouterClient
- Atualiza meta de conjunto de imagens no admin_datasets para 72 casos
</commit_message>
<xml_diff>
--- a/modelos_ia_previstos.xlsx
+++ b/modelos_ia_previstos.xlsx
@@ -2,100 +2,61 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="Modelos IA" sheetId="1" r:id="rId1"/>
+    <sheet name="Modelos Previstos" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
-</file>
-
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
-    <font>
-      <name val="Calibri"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <b/>
-      <name val="Calibri"/>
-      <sz val="11"/>
-    </font>
-  </fonts>
-  <fills count="2">
-    <fill>
-      <patternFill fillType="none"/>
-    </fill>
-    <fill>
-      <patternFill fillType="gray125"/>
-    </fill>
-  </fills>
-  <borders count="1">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-    </border>
-  </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-  </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-  </cellXfs>
-</styleSheet>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr" s="1">
+      <c r="A1" t="inlineStr">
         <is>
           <t>categoria</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr" s="1">
+      <c r="B1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr" s="1">
+      <c r="C1" t="inlineStr">
         <is>
           <t>nome_modelo</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr" s="1">
+      <c r="D1" t="inlineStr">
         <is>
           <t>identificador_tag</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr" s="1">
+      <c r="E1" t="inlineStr">
         <is>
           <t>provedor_runtime</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr" s="1">
+      <c r="F1" t="inlineStr">
         <is>
           <t>parametros</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr" s="1">
+      <c r="G1" t="inlineStr">
         <is>
           <t>quantizacao_dimensoes</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr" s="1">
+      <c r="H1" t="inlineStr">
         <is>
           <t>janela_contexto</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr" s="1">
+      <c r="I1" t="inlineStr">
         <is>
           <t>visao_local</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr" s="1">
+      <c r="J1" t="inlineStr">
         <is>
           <t>papel_no_projeto</t>
         </is>
@@ -109,17 +70,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>llama31-8b</t>
+          <t>llama32-11b-vision</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Llama 3.1 8B</t>
+          <t>Llama 3.2 11B Vision Instruct</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>llama3.1:8b</t>
+          <t>hf.co/leafspark/Llama-3.2-11B-Vision-Instruct-GGUF:Q8_0</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -129,27 +90,27 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>8B</t>
+          <t>11B</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Q4_0</t>
+          <t>Q8_0</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>8k/128k</t>
+          <t>128k</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>nao</t>
+          <t>sim</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Baseline de mercado / eficiencia geral</t>
+          <t>Multimodal nativo com visao e raciocinio avancado</t>
         </is>
       </c>
     </row>
@@ -171,7 +132,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>qwen2.5-vl:7b</t>
+          <t>hf.co/unsloth/Qwen2.5-VL-7B-Instruct-GGUF:UD-Q8_K_XL</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -186,7 +147,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Q4_K_M</t>
+          <t>UD-Q8_K_XL</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -213,17 +174,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>qwen3-14b-q4</t>
+          <t>qwen35-9b</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Qwen3 14B Q4_K_M</t>
+          <t>Qwen3.5 9B Q4_K_M</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>qwen3:14b-q4_K_M</t>
+          <t>qwen3.5:9b</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -233,7 +194,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>14B</t>
+          <t>9.7B</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -243,17 +204,17 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>32k</t>
+          <t>262k</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>nao</t>
+          <t>sim</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Teste de teto de capacidade em 16GB VRAM</t>
+          <t>Modelo denso moderno com raciocinio thinking nativo e visao local</t>
         </is>
       </c>
     </row>
@@ -265,17 +226,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>qwen3-14b-q5</t>
+          <t>qwen25-vl-3b</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Qwen3 14B Q5_K_M</t>
+          <t>Qwen2.5-VL 3B Instruct</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>qwen3:14b-q5_K_M</t>
+          <t>hf.co/unsloth/Qwen2.5-VL-3B-Instruct-GGUF:BF16</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -285,27 +246,27 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>14B</t>
+          <t>3B</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Q5_K_M</t>
+          <t>BF16</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>32k</t>
+          <t>32k/128k</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>nao</t>
+          <t>sim</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Teste de precisao x risco de contencao de VRAM</t>
+          <t>Modelo multimodal leve de altissima velocidade e visao local</t>
         </is>
       </c>
     </row>
@@ -317,17 +278,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>qwen3-8b-q5</t>
+          <t>deepseek-r1-distill-llama-8b-q8</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Qwen3 8B Q5_K_M</t>
+          <t>DeepSeek-R1-Distill-Llama-8B Q8_0</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>qwen3:8b-q5_K_M</t>
+          <t>hf.co/bartowski/DeepSeek-R1-Distill-Llama-8B-GGUF:Q8_0</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -342,12 +303,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Q5_K_M</t>
+          <t>Q8_0</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>32k</t>
+          <t>128k</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -357,7 +318,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Equilibrio entre latencia e fidelidade</t>
+          <t>Raciocinio profundo (reasoning) destilado do DeepSeek-R1 em alta precisao Q8_0</t>
         </is>
       </c>
     </row>
@@ -369,17 +330,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>qwen3-8b-q8</t>
+          <t>qwen35-9b-defiant-fable-mtp</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Qwen3 8B Q8_0</t>
+          <t>Qwen3.5-9B-The-Defiant-Fable-Uncensored-Heretic-NEO-IMATRIX-MAX-MTP</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>qwen3:8b-q8_0</t>
+          <t>hf.co/DavidAU/Qwen3.5-9B-The-Defiant-Fable-Uncensored-Heretic-NEO-IMATRIX-MAX-MTP-GGUF:Q8_0</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -389,7 +350,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>8B</t>
+          <t>9B</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -399,7 +360,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>32k</t>
+          <t>32k/128k</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -409,7 +370,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Teste de alta precisao de quantizacao (8-bit)</t>
+          <t>Raciocinio avancado com suporte a speculative decoding MTP</t>
         </is>
       </c>
     </row>
@@ -421,17 +382,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>phi4-mini</t>
+          <t>phi4-mini-bf16</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Phi-4-mini</t>
+          <t>Phi-4-mini-instruct BF16</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>phi4-mini</t>
+          <t>hf.co/unsloth/Phi-4-mini-instruct-GGUF:BF16</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -446,12 +407,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Q4_K_M</t>
+          <t>BF16</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>16k</t>
+          <t>128k</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -461,7 +422,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Candidato ultra-rapido de baixa latencia</t>
+          <t>Candidato leve em maxima precisao BF16 sem quantizacao</t>
         </is>
       </c>
     </row>
@@ -473,17 +434,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>phi4</t>
+          <t>gemma3-gaia-4b-f16</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Phi-4</t>
+          <t>Gemma-3-Gaia-PT-BR-4b-it F16</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>phi4</t>
+          <t>hf.co/mradermacher/Gemma-3-Gaia-PT-BR-4b-it-GGUF:F16</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -493,27 +454,27 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>14B</t>
+          <t>4B</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Q4_K_M</t>
+          <t>F16</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>16k</t>
+          <t>128k</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>nao</t>
+          <t>sim</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Modelo compacto com forte capacidade logica</t>
+          <t>Especializado em PT-BR com visao local nativa em alta precisao F16</t>
         </is>
       </c>
     </row>
@@ -587,7 +548,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>gemma-4-E4B-it-GGUF:UD-Q8_K_XL</t>
+          <t>hf.co/unsloth/gemma-4-E4B-it-GGUF:UD-Q8_K_XL</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -889,17 +850,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>qwen25-vl-local</t>
+          <t>gemma3-gaia-vision-local</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Qwen2.5-VL 7B Instruct Vision</t>
+          <t>Gemma-3-Gaia-PT-BR-4b-it Local Vision</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>qwen2.5-vl:7b</t>
+          <t>hf.co/mradermacher/Gemma-3-Gaia-PT-BR-4b-it-GGUF:F16</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -909,17 +870,17 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>7B</t>
+          <t>4B</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Q4_K_M</t>
+          <t>F16</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>32k</t>
+          <t>128k</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -929,7 +890,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Descricao e classificacao de imagens no proprio hardware (Visao Local)</t>
+          <t>Descricao e classificacao de imagens no proprio hardware em PT-BR</t>
         </is>
       </c>
     </row>
@@ -941,37 +902,37 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>gemma4-vision-ext</t>
+          <t>qwen25-vl-local</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Gemma-4-31B Vision Externa</t>
+          <t>Qwen2.5-VL 7B Instruct Vision</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>google/gemma-4-31b-it:free</t>
+          <t>hf.co/unsloth/Qwen2.5-VL-7B-Instruct-GGUF:UD-Q8_K_XL</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>OpenRouter (Externo)</t>
+          <t>Ollama (Local)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>31B</t>
+          <t>7B</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>API</t>
+          <t>UD-Q8_K_XL</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>8k</t>
+          <t>32k</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -981,7 +942,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Fallback externo (EXTERNAL_VISION_MODEL_NAME)</t>
+          <t>Descricao e classificacao de imagens no proprio hardware (Visao Local)</t>
         </is>
       </c>
     </row>
@@ -993,37 +954,37 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>clip</t>
+          <t>qwen25-vl-3b-local</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>CLIP Image Embeddings</t>
+          <t>Qwen2.5-VL 3B Instruct Vision</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>sentence-transformers/clip-ViT-B-32</t>
+          <t>hf.co/unsloth/Qwen2.5-VL-3B-Instruct-GGUF:BF16</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Local (Qdrant)</t>
+          <t>Ollama (Local)</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>3B</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>512 dims</t>
+          <t>BF16</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>32k</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1033,81 +994,81 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Busca vetorial de catalogo por similaridade de imagem</t>
+          <t>Descricao e classificacao de imagens no proprio hardware (Visao Local)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Externo / Avaliacao</t>
+          <t>Visao e Imagem</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>lfm-judge</t>
+          <t>llama32-vision-local</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Liquid LFM 2.5 2.6B (Juiz)</t>
+          <t>Llama 3.2 11B Vision Instruct</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>liquid/lfm-2.5-2.6b:free</t>
+          <t>hf.co/leafspark/Llama-3.2-11B-Vision-Instruct-GGUF:Q8_0</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>OpenRouter (Externo)</t>
+          <t>Ollama (Local)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2.6B</t>
+          <t>11B</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>API</t>
+          <t>Q8_0</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>32k</t>
+          <t>128k</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>nao</t>
+          <t>sim</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>LLM-as-judge neutro para RAG e Injecao de Prompt</t>
+          <t>Descricao e classificacao de imagens no proprio hardware (Visao Local)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Externo / Avaliacao</t>
+          <t>Visao e Imagem</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>claude-haiku</t>
+          <t>gemma4-vision-ext</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Claude 3.5 Haiku</t>
+          <t>Gemma-4-31B Vision Externa</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>anthropic/claude-3.5-haiku</t>
+          <t>google/gemma-4-31b-it:free</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1117,7 +1078,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>31B</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1127,7 +1088,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>200k</t>
+          <t>8k</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1137,34 +1098,34 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Comparacao de latencia e escalonamento local x externo</t>
+          <t>Fallback externo (EXTERNAL_VISION_MODEL_NAME)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Externo / Avaliacao</t>
+          <t>Visao e Imagem</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>jev-system-one</t>
+          <t>clip</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>TypeSafe Jev</t>
+          <t>CLIP Image Embeddings</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>typesafe/jev-latest</t>
+          <t>sentence-transformers/clip-ViT-B-32</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>OpenRouter (System One)</t>
+          <t>Local (Qdrant)</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1174,7 +1135,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>API</t>
+          <t>512 dims</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1184,62 +1145,218 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>nao</t>
+          <t>sim</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Classificacao ultra-rapida de intencao e tom (&lt;10s)</t>
+          <t>Busca vetorial de catalogo por similaridade de imagem</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>Externo / Avaliacao</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>lfm-judge</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Liquid LFM 2.5 2.6B (Juiz)</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>liquid/lfm-2.5-2.6b:free</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>OpenRouter (Externo)</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>2.6B</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>32k</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>nao</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>LLM-as-judge neutro para RAG e Injecao de Prompt</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Externo / Avaliacao</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>claude-haiku</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Claude 3.5 Haiku</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>anthropic/claude-3.5-haiku</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>OpenRouter (Externo)</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>200k</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Comparacao de latencia e escalonamento local x externo</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Externo / Avaliacao</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>jev-system-one</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>TypeSafe Jev</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>typesafe/jev-latest</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>OpenRouter (System One)</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>nao</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Classificacao ultra-rapida de intencao e tom (&lt;10s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
           <t>Audio / STT</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>faster-whisper-small</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>faster-whisper small</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>small</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>Local (GPU CUDA)</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="F26" t="inlineStr">
         <is>
           <t>244M</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="G26" t="inlineStr">
         <is>
           <t>FP16</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="H26" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
+      <c r="I26" t="inlineStr">
         <is>
           <t>nao</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="J26" t="inlineStr">
         <is>
           <t>Transcricao local de audio na mesma GPU do SLM</t>
         </is>

</xml_diff>